<commit_message>
Versão preparada para fazer o 1º teste
</commit_message>
<xml_diff>
--- a/modelos/OdP's de cada odp.xlsx
+++ b/modelos/OdP's de cada odp.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F5D422C-9346-442A-8339-9164004B0EA8}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E9A9D16-9D8A-464E-8459-46F2CE1235DE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo" sheetId="1" r:id="rId1"/>
-    <sheet name="historico_modelo" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>DATA:</t>
   </si>
@@ -65,21 +64,9 @@
     <t>ODP´S DE CADA FUNCIONÁRIO</t>
   </si>
   <si>
-    <t>HISTÓRICO</t>
-  </si>
-  <si>
-    <t>DATA</t>
-  </si>
-  <si>
-    <t>HORA</t>
-  </si>
-  <si>
     <t>IDENTIFICADOR</t>
   </si>
   <si>
-    <t>ODP</t>
-  </si>
-  <si>
     <t>AÇÃO</t>
   </si>
   <si>
@@ -101,17 +88,17 @@
     <t>MÁQUINA</t>
   </si>
   <si>
-    <t>DATA DA PESAGEM</t>
-  </si>
-  <si>
     <t>OdP DA PESAGEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATA DA PESAGEM </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -153,20 +140,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -436,7 +409,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -445,9 +418,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -469,6 +439,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -544,20 +517,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -860,14 +827,14 @@
     <row r="3" spans="1:33" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="18"/>
       <c r="B3" s="19"/>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="11"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="10"/>
       <c r="G3" s="37"/>
       <c r="H3" s="38"/>
       <c r="I3" s="38"/>
@@ -914,68 +881,68 @@
     <row r="5" spans="1:33" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A5" s="22"/>
       <c r="B5" s="23"/>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="L5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="M5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="N5" s="5" t="s">
+      <c r="N5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="O5" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q5" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="R5" s="6" t="s">
+      <c r="O5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q5" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="S5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="T5" s="6" t="s">
+      <c r="R5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="W5" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="U5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="V5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="W5" s="7" t="s">
-        <v>21</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
@@ -1006,78 +973,4 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A88BC175-D680-46AF-B115-61DFC37BBD7C}">
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="1.42578125" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" customWidth="1"/>
-    <col min="3" max="4" width="13.140625" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" customWidth="1"/>
-    <col min="8" max="8" width="17.140625" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="40"/>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-    </row>
-    <row r="2" spans="1:9" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="40"/>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-    </row>
-    <row r="3" spans="1:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="40"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:I2"/>
-    <mergeCell ref="A3:B3"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>